<commit_message>
WIP: fee proposal outputs from running agents
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RKGFyarCMuMinKYL7AiBap
</commit_message>
<xml_diff>
--- a/FP/VP527469/Final/Part_B2-Returnable_Schedules-CQA_Engineer_JCE_FILLED_RevG.xlsx
+++ b/FP/VP527469/Final/Part_B2-Returnable_Schedules-CQA_Engineer_JCE_FILLED_RevG.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="214" uniqueCount="130">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="220" uniqueCount="133">
   <si>
     <t xml:space="preserve">CQA Engineer</t>
   </si>
@@ -223,6 +223,15 @@
     <t xml:space="preserve">Prepared and signed by JCE (CQA Engineer of record), reviewed and co-signed by the partner's senior landfill CQA engineer (PS3).</t>
   </si>
   <si>
+    <t xml:space="preserve">3.1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Associate Principal Engineer (S. Lotay, RPEQ, NER, Lotay Civil) - added line: independent review of the CQA Implementation Plan and CQA report, certification support</t>
+  </si>
+  <si>
+    <t xml:space="preserve">hr</t>
+  </si>
+  <si>
     <t xml:space="preserve">3A</t>
   </si>
   <si>
@@ -286,9 +295,6 @@
     <t xml:space="preserve">Lead CQA Engineer (J. Callen) $190/hr; site day (10 h) $1,900; Director review &amp; certification $200/hr; Project engineer/admin/travel $180/hr</t>
   </si>
   <si>
-    <t xml:space="preserve">hr</t>
-  </si>
-  <si>
     <t xml:space="preserve">4.2</t>
   </si>
   <si>
@@ -365,6 +371,9 @@
   </si>
   <si>
     <t xml:space="preserve">7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7.1</t>
   </si>
   <si>
     <t xml:space="preserve">7A</t>
@@ -868,7 +877,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:I89"/>
+  <dimension ref="A1:I91"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="7"/>
@@ -1521,41 +1530,41 @@
         <v>66</v>
       </c>
     </row>
-    <row r="36" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="10" t="s">
+    <row r="36" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="B36" s="11" t="s">
+      <c r="B36" s="12" t="s">
         <v>68</v>
       </c>
-      <c r="C36" s="10"/>
-      <c r="D36" s="10"/>
-      <c r="E36" s="10"/>
-      <c r="F36" s="10"/>
-      <c r="G36" s="10"/>
-      <c r="H36" s="10"/>
-      <c r="I36" s="10"/>
+      <c r="C36" s="5" t="n">
+        <v>16</v>
+      </c>
+      <c r="G36" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="H36" s="13" t="n">
+        <v>200</v>
+      </c>
+      <c r="I36" s="13" t="n">
+        <f aca="false">C36*H36</f>
+        <v>3200</v>
+      </c>
     </row>
     <row r="37" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="5" t="s">
-        <v>69</v>
-      </c>
-      <c r="B37" s="12" t="s">
+      <c r="A37" s="10" t="s">
         <v>70</v>
       </c>
-      <c r="C37" s="5" t="n">
-        <v>60</v>
-      </c>
-      <c r="G37" s="5" t="s">
+      <c r="B37" s="11" t="s">
         <v>71</v>
       </c>
-      <c r="H37" s="13" t="n">
-        <v>1430</v>
-      </c>
-      <c r="I37" s="13" t="n">
-        <f aca="false">C37*H37</f>
-        <v>85800</v>
-      </c>
+      <c r="C37" s="10"/>
+      <c r="D37" s="10"/>
+      <c r="E37" s="10"/>
+      <c r="F37" s="10"/>
+      <c r="G37" s="10"/>
+      <c r="H37" s="10"/>
+      <c r="I37" s="10"/>
     </row>
     <row r="38" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="5" t="s">
@@ -1565,46 +1574,46 @@
         <v>73</v>
       </c>
       <c r="C38" s="5" t="n">
-        <v>85</v>
+        <v>60</v>
       </c>
       <c r="G38" s="5" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="H38" s="13" t="n">
         <v>1430</v>
       </c>
       <c r="I38" s="13" t="n">
         <f aca="false">C38*H38</f>
-        <v>121550</v>
+        <v>85800</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="B39" s="12" t="s">
+        <v>76</v>
+      </c>
+      <c r="C39" s="5" t="n">
+        <v>85</v>
+      </c>
+      <c r="G39" s="5" t="s">
         <v>74</v>
       </c>
-      <c r="B39" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="C39" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="G39" s="5" t="s">
-        <v>29</v>
-      </c>
       <c r="H39" s="13" t="n">
-        <v>13200</v>
+        <v>1430</v>
       </c>
       <c r="I39" s="13" t="n">
         <f aca="false">C39*H39</f>
-        <v>13200</v>
+        <v>121550</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="5" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B40" s="12" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C40" s="5" t="n">
         <v>1</v>
@@ -1620,12 +1629,12 @@
         <v>13200</v>
       </c>
     </row>
-    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="41" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="5" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B41" s="12" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C41" s="5" t="n">
         <v>1</v>
@@ -1634,86 +1643,92 @@
         <v>29</v>
       </c>
       <c r="H41" s="13" t="n">
-        <v>30800</v>
+        <v>13200</v>
       </c>
       <c r="I41" s="13" t="n">
         <f aca="false">C41*H41</f>
+        <v>13200</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="B42" s="12" t="s">
+        <v>82</v>
+      </c>
+      <c r="C42" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="G42" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="H42" s="13" t="n">
         <v>30800</v>
-      </c>
-    </row>
-    <row r="42" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="5" t="s">
-        <v>80</v>
-      </c>
-      <c r="B42" s="12" t="s">
-        <v>81</v>
-      </c>
-      <c r="C42" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="G42" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="H42" s="13" t="n">
-        <v>41800</v>
       </c>
       <c r="I42" s="13" t="n">
         <f aca="false">C42*H42</f>
+        <v>30800</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="B43" s="12" t="s">
+        <v>84</v>
+      </c>
+      <c r="C43" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="G43" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="H43" s="13" t="n">
         <v>41800</v>
-      </c>
-    </row>
-    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="5" t="s">
-        <v>82</v>
-      </c>
-      <c r="B43" s="12" t="s">
-        <v>83</v>
-      </c>
-      <c r="C43" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="G43" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="H43" s="13" t="n">
-        <v>6600</v>
       </c>
       <c r="I43" s="13" t="n">
         <f aca="false">C43*H43</f>
+        <v>41800</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="B44" s="12" t="s">
+        <v>86</v>
+      </c>
+      <c r="C44" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="G44" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="H44" s="13" t="n">
         <v>6600</v>
       </c>
-    </row>
-    <row r="44" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="10" t="s">
-        <v>84</v>
-      </c>
-      <c r="B44" s="11" t="s">
-        <v>85</v>
-      </c>
-      <c r="C44" s="10"/>
-      <c r="D44" s="10"/>
-      <c r="E44" s="10"/>
-      <c r="F44" s="10"/>
-      <c r="G44" s="10"/>
-      <c r="H44" s="10"/>
-      <c r="I44" s="10"/>
+      <c r="I44" s="13" t="n">
+        <f aca="false">C44*H44</f>
+        <v>6600</v>
+      </c>
     </row>
     <row r="45" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="5" t="s">
-        <v>86</v>
-      </c>
-      <c r="B45" s="12" t="s">
+      <c r="A45" s="10" t="s">
         <v>87</v>
       </c>
-      <c r="G45" s="5" t="s">
+      <c r="B45" s="11" t="s">
         <v>88</v>
       </c>
-      <c r="H45" s="13" t="n">
-        <v>190</v>
-      </c>
-      <c r="I45" s="5"/>
-    </row>
-    <row r="46" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C45" s="10"/>
+      <c r="D45" s="10"/>
+      <c r="E45" s="10"/>
+      <c r="F45" s="10"/>
+      <c r="G45" s="10"/>
+      <c r="H45" s="10"/>
+      <c r="I45" s="10"/>
+    </row>
+    <row r="46" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="5" t="s">
         <v>89</v>
       </c>
@@ -1721,155 +1736,143 @@
         <v>90</v>
       </c>
       <c r="G46" s="5" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="H46" s="13" t="n">
+        <v>190</v>
+      </c>
+      <c r="I46" s="5"/>
+    </row>
+    <row r="47" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="5" t="s">
+        <v>91</v>
+      </c>
+      <c r="B47" s="12" t="s">
+        <v>92</v>
+      </c>
+      <c r="G47" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="H47" s="13" t="n">
         <v>1430</v>
       </c>
-      <c r="I46" s="5"/>
-    </row>
-    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H47" s="10" t="s">
-        <v>91</v>
-      </c>
-      <c r="I47" s="7" t="n">
-        <f aca="false">SUM(I14:I43)</f>
-        <v>450046.8</v>
-      </c>
-    </row>
-    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="8"/>
-      <c r="B49" s="9" t="s">
-        <v>92</v>
-      </c>
-      <c r="C49" s="8"/>
-      <c r="D49" s="8"/>
-      <c r="E49" s="8"/>
-      <c r="F49" s="8"/>
-      <c r="G49" s="8"/>
-      <c r="H49" s="8"/>
-      <c r="I49" s="8"/>
+      <c r="I47" s="5"/>
+    </row>
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="H48" s="10" t="s">
+        <v>93</v>
+      </c>
+      <c r="I48" s="7" t="n">
+        <f aca="false">SUM(I14:I44)</f>
+        <v>453246.8</v>
+      </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="10" t="s">
-        <v>93</v>
-      </c>
-      <c r="B50" s="11" t="s">
+      <c r="A50" s="8"/>
+      <c r="B50" s="9" t="s">
+        <v>94</v>
+      </c>
+      <c r="C50" s="8"/>
+      <c r="D50" s="8"/>
+      <c r="E50" s="8"/>
+      <c r="F50" s="8"/>
+      <c r="G50" s="8"/>
+      <c r="H50" s="8"/>
+      <c r="I50" s="8"/>
+    </row>
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A51" s="10" t="s">
+        <v>95</v>
+      </c>
+      <c r="B51" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="C50" s="10"/>
-      <c r="D50" s="10"/>
-      <c r="E50" s="10"/>
-      <c r="F50" s="10"/>
-      <c r="G50" s="10"/>
-      <c r="H50" s="10"/>
-      <c r="I50" s="10"/>
-    </row>
-    <row r="51" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="5" t="s">
-        <v>94</v>
-      </c>
-      <c r="B51" s="12" t="s">
+      <c r="C51" s="10"/>
+      <c r="D51" s="10"/>
+      <c r="E51" s="10"/>
+      <c r="F51" s="10"/>
+      <c r="G51" s="10"/>
+      <c r="H51" s="10"/>
+      <c r="I51" s="10"/>
+    </row>
+    <row r="52" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A52" s="5" t="s">
+        <v>96</v>
+      </c>
+      <c r="B52" s="12" t="s">
         <v>28</v>
       </c>
-      <c r="C51" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="D51" s="5" t="n">
+      <c r="C52" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D52" s="5" t="n">
         <v>50</v>
       </c>
-      <c r="E51" s="5" t="n">
+      <c r="E52" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="F51" s="5" t="n">
+      <c r="F52" s="5" t="n">
         <v>95</v>
       </c>
-      <c r="G51" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="H51" s="13" t="n">
-        <f aca="false">D51*$D$11+E51*$E$11+F51*$F$11</f>
+      <c r="G52" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="H52" s="13" t="n">
+        <f aca="false">D52*$D$11+E52*$E$11+F52*$F$11</f>
         <v>27400</v>
       </c>
-      <c r="I51" s="13" t="n">
-        <f aca="false">C51*H51</f>
+      <c r="I52" s="13" t="n">
+        <f aca="false">C52*H52</f>
         <v>27400</v>
       </c>
     </row>
-    <row r="52" customFormat="false" ht="37.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B52" s="14" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="53" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A53" s="5" t="s">
-        <v>96</v>
-      </c>
-      <c r="B53" s="12" t="s">
+    <row r="53" customFormat="false" ht="37.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B53" s="14" t="s">
         <v>97</v>
       </c>
-      <c r="C53" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="G53" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="H53" s="13" t="n">
+    </row>
+    <row r="54" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A54" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="B54" s="12" t="s">
+        <v>99</v>
+      </c>
+      <c r="C54" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="G54" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="H54" s="13" t="n">
         <v>9688</v>
       </c>
-      <c r="I53" s="13" t="n">
-        <f aca="false">C53*H53</f>
+      <c r="I54" s="13" t="n">
+        <f aca="false">C54*H54</f>
         <v>9688</v>
       </c>
     </row>
-    <row r="54" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A54" s="10" t="s">
-        <v>98</v>
-      </c>
-      <c r="B54" s="11" t="s">
+    <row r="55" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A55" s="10" t="s">
+        <v>100</v>
+      </c>
+      <c r="B55" s="11" t="s">
         <v>34</v>
       </c>
-      <c r="C54" s="10"/>
-      <c r="D54" s="10"/>
-      <c r="E54" s="10"/>
-      <c r="F54" s="10"/>
-      <c r="G54" s="10"/>
-      <c r="H54" s="10"/>
-      <c r="I54" s="10"/>
-    </row>
-    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A55" s="5" t="s">
-        <v>99</v>
-      </c>
-      <c r="B55" s="12" t="s">
-        <v>36</v>
-      </c>
-      <c r="C55" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="D55" s="5" t="n">
-        <v>13</v>
-      </c>
-      <c r="E55" s="5"/>
-      <c r="F55" s="5"/>
-      <c r="G55" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="H55" s="13" t="n">
-        <f aca="false">D55*$D$11+E55*$E$11+F55*$F$11</f>
-        <v>2470</v>
-      </c>
-      <c r="I55" s="13" t="n">
-        <f aca="false">C55*H55</f>
-        <v>2470</v>
-      </c>
+      <c r="C55" s="10"/>
+      <c r="D55" s="10"/>
+      <c r="E55" s="10"/>
+      <c r="F55" s="10"/>
+      <c r="G55" s="10"/>
+      <c r="H55" s="10"/>
+      <c r="I55" s="10"/>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="5" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="B56" s="12" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="C56" s="5" t="n">
         <v>1</v>
@@ -1893,72 +1896,72 @@
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="5" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B57" s="12" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C57" s="5" t="n">
         <v>1</v>
       </c>
       <c r="D57" s="5" t="n">
-        <v>22</v>
-      </c>
-      <c r="E57" s="5" t="n">
-        <v>1</v>
-      </c>
+        <v>13</v>
+      </c>
+      <c r="E57" s="5"/>
       <c r="F57" s="5"/>
       <c r="G57" s="5" t="s">
         <v>29</v>
       </c>
       <c r="H57" s="13" t="n">
         <f aca="false">D57*$D$11+E57*$E$11+F57*$F$11</f>
-        <v>4380</v>
+        <v>2470</v>
       </c>
       <c r="I57" s="13" t="n">
         <f aca="false">C57*H57</f>
-        <v>4380</v>
+        <v>2470</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="5" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B58" s="12" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="C58" s="5" t="n">
         <v>1</v>
       </c>
       <c r="D58" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="E58" s="5"/>
+        <v>22</v>
+      </c>
+      <c r="E58" s="5" t="n">
+        <v>1</v>
+      </c>
       <c r="F58" s="5"/>
       <c r="G58" s="5" t="s">
         <v>29</v>
       </c>
       <c r="H58" s="13" t="n">
         <f aca="false">D58*$D$11+E58*$E$11+F58*$F$11</f>
-        <v>760</v>
+        <v>4380</v>
       </c>
       <c r="I58" s="13" t="n">
         <f aca="false">C58*H58</f>
-        <v>760</v>
+        <v>4380</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="5" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B59" s="12" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="C59" s="5" t="n">
         <v>1</v>
       </c>
       <c r="D59" s="5" t="n">
-        <v>18</v>
+        <v>4</v>
       </c>
       <c r="E59" s="5"/>
       <c r="F59" s="5"/>
@@ -1967,81 +1970,81 @@
       </c>
       <c r="H59" s="13" t="n">
         <f aca="false">D59*$D$11+E59*$E$11+F59*$F$11</f>
-        <v>3420</v>
+        <v>760</v>
       </c>
       <c r="I59" s="13" t="n">
         <f aca="false">C59*H59</f>
-        <v>3420</v>
+        <v>760</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="5" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B60" s="12" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="C60" s="5" t="n">
         <v>1</v>
       </c>
       <c r="D60" s="5" t="n">
-        <v>46</v>
-      </c>
-      <c r="E60" s="5" t="n">
-        <v>3</v>
-      </c>
+        <v>18</v>
+      </c>
+      <c r="E60" s="5"/>
       <c r="F60" s="5"/>
       <c r="G60" s="5" t="s">
         <v>29</v>
       </c>
       <c r="H60" s="13" t="n">
         <f aca="false">D60*$D$11+E60*$E$11+F60*$F$11</f>
-        <v>9340</v>
+        <v>3420</v>
       </c>
       <c r="I60" s="13" t="n">
         <f aca="false">C60*H60</f>
-        <v>9340</v>
+        <v>3420</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="5" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B61" s="12" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="C61" s="5" t="n">
         <v>1</v>
       </c>
       <c r="D61" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="E61" s="5"/>
+        <v>46</v>
+      </c>
+      <c r="E61" s="5" t="n">
+        <v>3</v>
+      </c>
       <c r="F61" s="5"/>
       <c r="G61" s="5" t="s">
         <v>29</v>
       </c>
       <c r="H61" s="13" t="n">
         <f aca="false">D61*$D$11+E61*$E$11+F61*$F$11</f>
-        <v>760</v>
+        <v>9340</v>
       </c>
       <c r="I61" s="13" t="n">
         <f aca="false">C61*H61</f>
-        <v>760</v>
+        <v>9340</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="5" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B62" s="12" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C62" s="5" t="n">
         <v>1</v>
       </c>
       <c r="D62" s="5" t="n">
-        <v>16</v>
+        <v>4</v>
       </c>
       <c r="E62" s="5"/>
       <c r="F62" s="5"/>
@@ -2050,19 +2053,19 @@
       </c>
       <c r="H62" s="13" t="n">
         <f aca="false">D62*$D$11+E62*$E$11+F62*$F$11</f>
-        <v>3040</v>
+        <v>760</v>
       </c>
       <c r="I62" s="13" t="n">
         <f aca="false">C62*H62</f>
-        <v>3040</v>
+        <v>760</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="5" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B63" s="12" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="C63" s="5" t="n">
         <v>1</v>
@@ -2070,55 +2073,55 @@
       <c r="D63" s="5" t="n">
         <v>16</v>
       </c>
-      <c r="E63" s="5" t="n">
-        <v>1</v>
-      </c>
+      <c r="E63" s="5"/>
       <c r="F63" s="5"/>
       <c r="G63" s="5" t="s">
         <v>29</v>
       </c>
       <c r="H63" s="13" t="n">
         <f aca="false">D63*$D$11+E63*$E$11+F63*$F$11</f>
-        <v>3240</v>
+        <v>3040</v>
       </c>
       <c r="I63" s="13" t="n">
         <f aca="false">C63*H63</f>
-        <v>3240</v>
+        <v>3040</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="5" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B64" s="12" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="C64" s="5" t="n">
         <v>1</v>
       </c>
       <c r="D64" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="E64" s="5"/>
+        <v>16</v>
+      </c>
+      <c r="E64" s="5" t="n">
+        <v>1</v>
+      </c>
       <c r="F64" s="5"/>
       <c r="G64" s="5" t="s">
         <v>29</v>
       </c>
       <c r="H64" s="13" t="n">
         <f aca="false">D64*$D$11+E64*$E$11+F64*$F$11</f>
-        <v>760</v>
+        <v>3240</v>
       </c>
       <c r="I64" s="13" t="n">
         <f aca="false">C64*H64</f>
-        <v>760</v>
+        <v>3240</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="5" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B65" s="12" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="C65" s="5" t="n">
         <v>1</v>
@@ -2142,16 +2145,16 @@
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="5" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="B66" s="12" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="C66" s="5" t="n">
         <v>1</v>
       </c>
       <c r="D66" s="5" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E66" s="5"/>
       <c r="F66" s="5"/>
@@ -2160,19 +2163,19 @@
       </c>
       <c r="H66" s="13" t="n">
         <f aca="false">D66*$D$11+E66*$E$11+F66*$F$11</f>
-        <v>570</v>
+        <v>760</v>
       </c>
       <c r="I66" s="13" t="n">
         <f aca="false">C66*H66</f>
-        <v>570</v>
+        <v>760</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="5" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="B67" s="12" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="C67" s="5" t="n">
         <v>1</v>
@@ -2196,16 +2199,16 @@
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="5" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="B68" s="12" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="C68" s="5" t="n">
         <v>1</v>
       </c>
       <c r="D68" s="5" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="E68" s="5"/>
       <c r="F68" s="5"/>
@@ -2214,159 +2217,165 @@
       </c>
       <c r="H68" s="13" t="n">
         <f aca="false">D68*$D$11+E68*$E$11+F68*$F$11</f>
-        <v>1140</v>
+        <v>570</v>
       </c>
       <c r="I68" s="13" t="n">
         <f aca="false">C68*H68</f>
+        <v>570</v>
+      </c>
+    </row>
+    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A69" s="5" t="s">
+        <v>114</v>
+      </c>
+      <c r="B69" s="12" t="s">
+        <v>62</v>
+      </c>
+      <c r="C69" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D69" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="E69" s="5"/>
+      <c r="F69" s="5"/>
+      <c r="G69" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="H69" s="13" t="n">
+        <f aca="false">D69*$D$11+E69*$E$11+F69*$F$11</f>
         <v>1140</v>
       </c>
-    </row>
-    <row r="69" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B69" s="14" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A70" s="5" t="s">
-        <v>114</v>
-      </c>
-      <c r="B70" s="12" t="s">
+      <c r="I69" s="13" t="n">
+        <f aca="false">C69*H69</f>
+        <v>1140</v>
+      </c>
+    </row>
+    <row r="70" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B70" s="14" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A71" s="5" t="s">
+        <v>116</v>
+      </c>
+      <c r="B71" s="12" t="s">
         <v>65</v>
       </c>
-      <c r="C70" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="D70" s="5" t="n">
+      <c r="C71" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D71" s="5" t="n">
         <v>40</v>
       </c>
-      <c r="E70" s="5" t="n">
+      <c r="E71" s="5" t="n">
         <v>8</v>
       </c>
-      <c r="F70" s="5" t="n">
+      <c r="F71" s="5" t="n">
         <v>10</v>
       </c>
-      <c r="G70" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="H70" s="13" t="n">
-        <f aca="false">D70*$D$11+E70*$E$11+F70*$F$11</f>
+      <c r="G71" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="H71" s="13" t="n">
+        <f aca="false">D71*$D$11+E71*$E$11+F71*$F$11</f>
         <v>11000</v>
       </c>
-      <c r="I70" s="13" t="n">
-        <f aca="false">C70*H70</f>
+      <c r="I71" s="13" t="n">
+        <f aca="false">C71*H71</f>
         <v>11000</v>
       </c>
     </row>
-    <row r="71" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B71" s="14" t="s">
+    <row r="72" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B72" s="14" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="72" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A72" s="10" t="s">
-        <v>115</v>
-      </c>
-      <c r="B72" s="11" t="s">
+    <row r="73" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A73" s="5" t="s">
+        <v>117</v>
+      </c>
+      <c r="B73" s="12" t="s">
         <v>68</v>
       </c>
-      <c r="C72" s="10"/>
-      <c r="D72" s="10"/>
-      <c r="E72" s="10"/>
-      <c r="F72" s="10"/>
-      <c r="G72" s="10"/>
-      <c r="H72" s="10"/>
-      <c r="I72" s="10"/>
-    </row>
-    <row r="73" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A73" s="5" t="s">
-        <v>116</v>
-      </c>
-      <c r="B73" s="12" t="s">
-        <v>70</v>
-      </c>
       <c r="C73" s="5" t="n">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="G73" s="5" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="H73" s="13" t="n">
-        <v>1430</v>
+        <v>200</v>
       </c>
       <c r="I73" s="13" t="n">
         <f aca="false">C73*H73</f>
-        <v>42900</v>
+        <v>2000</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A74" s="5" t="s">
-        <v>117</v>
-      </c>
-      <c r="B74" s="12" t="s">
-        <v>73</v>
-      </c>
-      <c r="C74" s="5" t="n">
-        <v>50</v>
-      </c>
-      <c r="G74" s="5" t="s">
+      <c r="A74" s="10" t="s">
+        <v>118</v>
+      </c>
+      <c r="B74" s="11" t="s">
         <v>71</v>
       </c>
-      <c r="H74" s="13" t="n">
-        <v>1430</v>
-      </c>
-      <c r="I74" s="13" t="n">
-        <f aca="false">C74*H74</f>
-        <v>71500</v>
-      </c>
+      <c r="C74" s="10"/>
+      <c r="D74" s="10"/>
+      <c r="E74" s="10"/>
+      <c r="F74" s="10"/>
+      <c r="G74" s="10"/>
+      <c r="H74" s="10"/>
+      <c r="I74" s="10"/>
     </row>
     <row r="75" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="5" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B75" s="12" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="C75" s="5" t="n">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="G75" s="5" t="s">
-        <v>29</v>
+        <v>74</v>
       </c>
       <c r="H75" s="13" t="n">
-        <v>7700</v>
+        <v>1430</v>
       </c>
       <c r="I75" s="13" t="n">
         <f aca="false">C75*H75</f>
-        <v>7700</v>
+        <v>42900</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="5" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="B76" s="12" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C76" s="5" t="n">
-        <v>1</v>
+        <v>50</v>
       </c>
       <c r="G76" s="5" t="s">
-        <v>29</v>
+        <v>74</v>
       </c>
       <c r="H76" s="13" t="n">
-        <v>6600</v>
+        <v>1430</v>
       </c>
       <c r="I76" s="13" t="n">
         <f aca="false">C76*H76</f>
-        <v>6600</v>
-      </c>
-    </row>
-    <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>71500</v>
+      </c>
+    </row>
+    <row r="77" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="5" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="B77" s="12" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C77" s="5" t="n">
         <v>1</v>
@@ -2375,19 +2384,19 @@
         <v>29</v>
       </c>
       <c r="H77" s="13" t="n">
-        <v>15400</v>
+        <v>7700</v>
       </c>
       <c r="I77" s="13" t="n">
         <f aca="false">C77*H77</f>
-        <v>15400</v>
+        <v>7700</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="5" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="B78" s="12" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C78" s="5" t="n">
         <v>1</v>
@@ -2396,19 +2405,19 @@
         <v>29</v>
       </c>
       <c r="H78" s="13" t="n">
-        <v>17600</v>
+        <v>6600</v>
       </c>
       <c r="I78" s="13" t="n">
         <f aca="false">C78*H78</f>
-        <v>17600</v>
+        <v>6600</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="5" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="B79" s="12" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C79" s="5" t="n">
         <v>1</v>
@@ -2417,97 +2426,139 @@
         <v>29</v>
       </c>
       <c r="H79" s="13" t="n">
-        <v>3300</v>
+        <v>15400</v>
       </c>
       <c r="I79" s="13" t="n">
         <f aca="false">C79*H79</f>
+        <v>15400</v>
+      </c>
+    </row>
+    <row r="80" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A80" s="5" t="s">
+        <v>124</v>
+      </c>
+      <c r="B80" s="12" t="s">
+        <v>84</v>
+      </c>
+      <c r="C80" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="G80" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="H80" s="13" t="n">
+        <v>17600</v>
+      </c>
+      <c r="I80" s="13" t="n">
+        <f aca="false">C80*H80</f>
+        <v>17600</v>
+      </c>
+    </row>
+    <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A81" s="5" t="s">
+        <v>125</v>
+      </c>
+      <c r="B81" s="12" t="s">
+        <v>86</v>
+      </c>
+      <c r="C81" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="G81" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="H81" s="13" t="n">
         <v>3300</v>
       </c>
-    </row>
-    <row r="80" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A80" s="10" t="s">
-        <v>123</v>
-      </c>
-      <c r="B80" s="11" t="s">
-        <v>85</v>
-      </c>
-      <c r="C80" s="10"/>
-      <c r="D80" s="10"/>
-      <c r="E80" s="10"/>
-      <c r="F80" s="10"/>
-      <c r="G80" s="10"/>
-      <c r="H80" s="10"/>
-      <c r="I80" s="10"/>
-    </row>
-    <row r="81" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A81" s="5" t="s">
-        <v>124</v>
-      </c>
-      <c r="B81" s="12" t="s">
-        <v>87</v>
-      </c>
-      <c r="G81" s="5" t="s">
+      <c r="I81" s="13" t="n">
+        <f aca="false">C81*H81</f>
+        <v>3300</v>
+      </c>
+    </row>
+    <row r="82" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A82" s="10" t="s">
+        <v>126</v>
+      </c>
+      <c r="B82" s="11" t="s">
         <v>88</v>
       </c>
-      <c r="H81" s="13" t="n">
+      <c r="C82" s="10"/>
+      <c r="D82" s="10"/>
+      <c r="E82" s="10"/>
+      <c r="F82" s="10"/>
+      <c r="G82" s="10"/>
+      <c r="H82" s="10"/>
+      <c r="I82" s="10"/>
+    </row>
+    <row r="83" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A83" s="5" t="s">
+        <v>127</v>
+      </c>
+      <c r="B83" s="12" t="s">
+        <v>90</v>
+      </c>
+      <c r="G83" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="H83" s="13" t="n">
         <v>190</v>
       </c>
-      <c r="I81" s="5"/>
-    </row>
-    <row r="82" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A82" s="5" t="s">
-        <v>125</v>
-      </c>
-      <c r="B82" s="12" t="s">
-        <v>90</v>
-      </c>
-      <c r="G82" s="5" t="s">
-        <v>71</v>
-      </c>
-      <c r="H82" s="13" t="n">
+      <c r="I83" s="5"/>
+    </row>
+    <row r="84" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A84" s="5" t="s">
+        <v>128</v>
+      </c>
+      <c r="B84" s="12" t="s">
+        <v>92</v>
+      </c>
+      <c r="G84" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="H84" s="13" t="n">
         <v>1430</v>
       </c>
-      <c r="I82" s="5"/>
-    </row>
-    <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H83" s="10" t="s">
-        <v>91</v>
-      </c>
-      <c r="I83" s="7" t="n">
-        <f aca="false">SUM(I50:I79)</f>
-        <v>246768</v>
-      </c>
+      <c r="I84" s="5"/>
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H85" s="10" t="s">
-        <v>126</v>
+        <v>93</v>
       </c>
       <c r="I85" s="7" t="n">
-        <f aca="false">I47+I83</f>
-        <v>696814.8</v>
-      </c>
-    </row>
-    <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H86" s="10" t="s">
-        <v>127</v>
-      </c>
-      <c r="I86" s="15" t="n">
-        <f aca="false">ROUND(I85*0.1,2)</f>
-        <v>69681.48</v>
+        <f aca="false">SUM(I51:I81)</f>
+        <v>248768</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H87" s="10" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="I87" s="7" t="n">
-        <f aca="false">I85+I86</f>
-        <v>766496.28</v>
-      </c>
-    </row>
-    <row r="89" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B89" s="16" t="s">
-        <v>129</v>
+        <f aca="false">I48+I85</f>
+        <v>702014.8</v>
+      </c>
+    </row>
+    <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="H88" s="10" t="s">
+        <v>130</v>
+      </c>
+      <c r="I88" s="15" t="n">
+        <f aca="false">ROUND(I87*0.1,2)</f>
+        <v>70201.48</v>
+      </c>
+    </row>
+    <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="H89" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="I89" s="7" t="n">
+        <f aca="false">I87+I88</f>
+        <v>772216.28</v>
+      </c>
+    </row>
+    <row r="91" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B91" s="16" t="s">
+        <v>132</v>
       </c>
     </row>
   </sheetData>

</xml_diff>